<commit_message>
Finalization of Data Collection Pre-Analysis Push
</commit_message>
<xml_diff>
--- a/Farm Soils Data.xlsx
+++ b/Farm Soils Data.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://princetonu-my.sharepoint.com/personal/cg3403_princeton_edu/Documents/Undergraduate Research/Thesis Files/Thesis Rmd Doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1835" documentId="11_F25DC773A252ABDACC1048EB41DB448A5ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D002BF18-488B-4409-8D9A-9FE48655C303}"/>
+  <xr:revisionPtr revIDLastSave="2361" documentId="11_F25DC773A252ABDACC1048EB41DB448A5ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78957F7A-7803-43E8-8B02-49C4480BC9AA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="884" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="8100" windowWidth="19420" windowHeight="10300" tabRatio="884" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Characterization" sheetId="1" r:id="rId1"/>
     <sheet name="Oven Drying &amp; Combustion" sheetId="2" r:id="rId2"/>
     <sheet name="Trial Metadata" sheetId="7" r:id="rId3"/>
-    <sheet name="Soil Samples for Rutgers" sheetId="8" r:id="rId4"/>
-    <sheet name="Soil Sample Management" sheetId="6" r:id="rId5"/>
-    <sheet name="H Calibration" sheetId="4" r:id="rId6"/>
-    <sheet name="incomplete 01-28-26 Soy-UD" sheetId="5" r:id="rId7"/>
+    <sheet name="DNA Samples for Sequencing" sheetId="9" r:id="rId4"/>
+    <sheet name="Soil Samples for Rutgers" sheetId="8" r:id="rId5"/>
+    <sheet name="Soil Sample Management" sheetId="6" r:id="rId6"/>
+    <sheet name="H Calibration" sheetId="4" r:id="rId7"/>
+    <sheet name="incomplete 01-28-26 Soy-UD" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="265">
   <si>
     <t>Soybean Undisturbed</t>
   </si>
@@ -611,9 +612,6 @@
     <t>WP may be wrong, number slipped mind (but I think it was -19.something)</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
-  </si>
-  <si>
     <t>FGF-FBW-15-1</t>
   </si>
   <si>
@@ -648,16 +646,210 @@
   </si>
   <si>
     <t>FGF-SUN-25-3</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Sample # (on Cap)</t>
+  </si>
+  <si>
+    <t>FGF-RM-20-1</t>
+  </si>
+  <si>
+    <t>FGF-RM-20-2</t>
+  </si>
+  <si>
+    <t>FGF-RM-20-3</t>
+  </si>
+  <si>
+    <t>FGF-SF-20-1</t>
+  </si>
+  <si>
+    <t>FGF-SF-20-2</t>
+  </si>
+  <si>
+    <t>FGF-SF-20-3</t>
+  </si>
+  <si>
+    <t>FGF-OR-20-1</t>
+  </si>
+  <si>
+    <t>FGF-OR-20-2</t>
+  </si>
+  <si>
+    <t>FGF-OR-20-3</t>
+  </si>
+  <si>
+    <t>FGF-SOD-20-1</t>
+  </si>
+  <si>
+    <t>FGF-SOD-20-2</t>
+  </si>
+  <si>
+    <t>FGF-SOD-20-3</t>
+  </si>
+  <si>
+    <t>MF-AS-20-1</t>
+  </si>
+  <si>
+    <t>MF-AS-20-2</t>
+  </si>
+  <si>
+    <t>MF-AS-20-3</t>
+  </si>
+  <si>
+    <t>FGF-BW-20-1</t>
+  </si>
+  <si>
+    <t>FGF-BW-20-2</t>
+  </si>
+  <si>
+    <t>FGF-BW-20-3</t>
+  </si>
+  <si>
+    <t>MF-CH-20-1</t>
+  </si>
+  <si>
+    <t>MF-CH-20-2</t>
+  </si>
+  <si>
+    <t>MF-CH-20-3</t>
+  </si>
+  <si>
+    <t>Soy-UD-15-3</t>
+  </si>
+  <si>
+    <t>Soy-UD-25-1</t>
+  </si>
+  <si>
+    <t>Soy-UD-25-2</t>
+  </si>
+  <si>
+    <t>Soy-UD-25-3</t>
+  </si>
+  <si>
+    <t>Soy-C-15-1</t>
+  </si>
+  <si>
+    <t>Soy-C-15-2</t>
+  </si>
+  <si>
+    <t>Soy-C-15-3</t>
+  </si>
+  <si>
+    <t>Soy-C-25-1</t>
+  </si>
+  <si>
+    <t>Soy-C-25-2</t>
+  </si>
+  <si>
+    <t>Soy-C-25-3</t>
+  </si>
+  <si>
+    <t>FGF-CO-20-1</t>
+  </si>
+  <si>
+    <t>FGF-CO-20-2</t>
+  </si>
+  <si>
+    <t>FGF-CO-20-3</t>
+  </si>
+  <si>
+    <t>FGF-CO-15-1</t>
+  </si>
+  <si>
+    <t>FGF-CO-15-2</t>
+  </si>
+  <si>
+    <t>FGF-CO-15-3</t>
+  </si>
+  <si>
+    <t>FGF-CO-25-1</t>
+  </si>
+  <si>
+    <t>FGF-CO-25-2</t>
+  </si>
+  <si>
+    <t>FGF-CO-25-3</t>
+  </si>
+  <si>
+    <t>Sample Name Underscores</t>
+  </si>
+  <si>
+    <t>Wrong name in nanodrop:</t>
+  </si>
+  <si>
+    <t>Labelled as second MF-CH-20-2</t>
+  </si>
+  <si>
+    <t>Labelled 25-1</t>
+  </si>
+  <si>
+    <t>Realized here I had not been wiping top mount of nanodrop</t>
+  </si>
+  <si>
+    <t>174.5 upon redo</t>
+  </si>
+  <si>
+    <t>2nd MF-20-2 is this one - got a replicate on accident</t>
+  </si>
+  <si>
+    <t>216.8 upon redo</t>
+  </si>
+  <si>
+    <t>63.2 Upon redo</t>
+  </si>
+  <si>
+    <t>133.9 redo</t>
+  </si>
+  <si>
+    <t>450.8 on redo</t>
+  </si>
+  <si>
+    <t>57.7 redo</t>
+  </si>
+  <si>
+    <t>287.7 redo</t>
+  </si>
+  <si>
+    <t>147.3 redo, 141.1 redo 2, 137.3 redo 3</t>
+  </si>
+  <si>
+    <t>234.5 redo</t>
+  </si>
+  <si>
+    <t>462.5 redo</t>
+  </si>
+  <si>
+    <t>758.3 upon redo, 596.4 redo again, 619.7 redo again</t>
+  </si>
+  <si>
+    <t>0;5014</t>
+  </si>
+  <si>
+    <t>739.2 redo, 1138.1 redo again, 641.4 redo again</t>
+  </si>
+  <si>
+    <t>554.5 redo, 553.1 redo again</t>
+  </si>
+  <si>
+    <t>*OLD* NanoDrop DNA conc (ng/uL)</t>
+  </si>
+  <si>
+    <t>Correct NanoDrop DNA Conc (ng/ul)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yy;@"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -708,7 +900,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -725,6 +917,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1799,10 +1993,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4433,7 +4623,7 @@
         <v>46050</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E43" si="0">_xlfn.DAYS(D4,C4)</f>
+        <f t="shared" ref="E4:E62" si="0">_xlfn.DAYS(D4,C4)</f>
         <v>14</v>
       </c>
       <c r="F4" s="2">
@@ -6443,16 +6633,44 @@
       <c r="C44" s="4">
         <v>46098</v>
       </c>
-      <c r="D44" s="4"/>
+      <c r="D44" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F44" s="2">
         <f>2.0083-0.002</f>
         <v>2.0063000000000004</v>
       </c>
-      <c r="J44" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="M44" s="9"/>
-      <c r="N44" s="8"/>
+      <c r="G44" s="2">
+        <v>0.50339999999999996</v>
+      </c>
+      <c r="H44" s="3">
+        <v>-23.1</v>
+      </c>
+      <c r="I44" s="2">
+        <v>10.0167</v>
+      </c>
+      <c r="J44" s="2">
+        <v>10.5594</v>
+      </c>
+      <c r="K44" s="2">
+        <v>10.5412</v>
+      </c>
+      <c r="L44" s="2">
+        <f t="shared" ref="L44:L61" si="3">(J44-K44)/(K44-I44)</f>
+        <v>3.4699714013346469E-2</v>
+      </c>
+      <c r="M44" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B44, Characterization!A:A, 0))*L44/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B44, Characterization!A:A, 0))*0.01)</f>
+        <v>9.9036138313546546E-2</v>
+      </c>
+      <c r="N44" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B44, Characterization!A:A, 0))*F44</f>
+        <v>8.0068814235591521E-2</v>
+      </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
@@ -6464,13 +6682,44 @@
       <c r="C45" s="4">
         <v>46098</v>
       </c>
-      <c r="D45" s="4"/>
+      <c r="D45" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F45" s="2">
         <f>2.0048-0.0029</f>
         <v>2.0019</v>
       </c>
-      <c r="M45" s="9"/>
-      <c r="N45" s="8"/>
+      <c r="G45" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H45" s="3">
+        <v>-12.85</v>
+      </c>
+      <c r="I45" s="2">
+        <v>10.873699999999999</v>
+      </c>
+      <c r="J45" s="2">
+        <v>11.383599999999999</v>
+      </c>
+      <c r="K45" s="2">
+        <v>11.363</v>
+      </c>
+      <c r="L45" s="2">
+        <f t="shared" si="3"/>
+        <v>4.2100960555896072E-2</v>
+      </c>
+      <c r="M45" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B45, Characterization!A:A, 0))*L45/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B45, Characterization!A:A, 0))*0.01)</f>
+        <v>0.12015996878657788</v>
+      </c>
+      <c r="N45" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B45, Characterization!A:A, 0))*F45</f>
+        <v>7.9893215978782156E-2</v>
+      </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
@@ -6482,13 +6731,44 @@
       <c r="C46" s="4">
         <v>46098</v>
       </c>
-      <c r="D46" s="4"/>
+      <c r="D46" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F46" s="2">
         <f>2.0052-0.0021</f>
         <v>2.0030999999999999</v>
       </c>
-      <c r="M46" s="9"/>
-      <c r="N46" s="8"/>
+      <c r="G46" s="2">
+        <v>0.5141</v>
+      </c>
+      <c r="H46" s="3">
+        <v>-23.88</v>
+      </c>
+      <c r="I46" s="2">
+        <v>10.099500000000001</v>
+      </c>
+      <c r="J46" s="2">
+        <v>10.6052</v>
+      </c>
+      <c r="K46" s="2">
+        <v>10.588900000000001</v>
+      </c>
+      <c r="L46" s="2">
+        <f t="shared" si="3"/>
+        <v>3.3306089088678631E-2</v>
+      </c>
+      <c r="M46" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B46, Characterization!A:A, 0))*L46/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B46, Characterization!A:A, 0))*0.01)</f>
+        <v>9.5058606085369562E-2</v>
+      </c>
+      <c r="N46" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B46, Characterization!A:A, 0))*F46</f>
+        <v>7.9941106412457427E-2</v>
+      </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
@@ -6500,13 +6780,44 @@
       <c r="C47" s="4">
         <v>46098</v>
       </c>
-      <c r="D47" s="4"/>
+      <c r="D47" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F47" s="2">
         <f>2.0041-0.0034</f>
         <v>2.0007000000000001</v>
       </c>
-      <c r="M47" s="9"/>
-      <c r="N47" s="8"/>
+      <c r="G47" s="2">
+        <v>0.49740000000000001</v>
+      </c>
+      <c r="H47" s="3">
+        <v>-5.24</v>
+      </c>
+      <c r="I47" s="2">
+        <v>10.8667</v>
+      </c>
+      <c r="J47" s="2">
+        <v>11.4329</v>
+      </c>
+      <c r="K47" s="2">
+        <v>11.402200000000001</v>
+      </c>
+      <c r="L47" s="2">
+        <f t="shared" si="3"/>
+        <v>5.7329598506068093E-2</v>
+      </c>
+      <c r="M47" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B47, Characterization!A:A, 0))*L47/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B47, Characterization!A:A, 0))*0.01)</f>
+        <v>0.16362388591800064</v>
+      </c>
+      <c r="N47" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B47, Characterization!A:A, 0))*F47</f>
+        <v>7.9845325545106885E-2</v>
+      </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
@@ -6518,13 +6829,44 @@
       <c r="C48" s="4">
         <v>46098</v>
       </c>
-      <c r="D48" s="4"/>
+      <c r="D48" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F48" s="2">
         <f>2.0013-0.0017</f>
         <v>1.9996</v>
       </c>
-      <c r="M48" s="9"/>
-      <c r="N48" s="8"/>
+      <c r="G48" s="2">
+        <v>0.50519999999999998</v>
+      </c>
+      <c r="H48" s="3">
+        <v>-5.61</v>
+      </c>
+      <c r="I48" s="2">
+        <v>10.1945</v>
+      </c>
+      <c r="J48" s="2">
+        <v>10.7476</v>
+      </c>
+      <c r="K48" s="2">
+        <v>10.716200000000001</v>
+      </c>
+      <c r="L48" s="2">
+        <f t="shared" si="3"/>
+        <v>6.01878474218892E-2</v>
+      </c>
+      <c r="M48" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B48, Characterization!A:A, 0))*L48/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B48, Characterization!A:A, 0))*0.01)</f>
+        <v>0.17178158816456462</v>
+      </c>
+      <c r="N48" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B48, Characterization!A:A, 0))*F48</f>
+        <v>7.9801425980904533E-2</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
@@ -6536,17 +6878,48 @@
       <c r="C49" s="4">
         <v>46098</v>
       </c>
-      <c r="D49" s="4"/>
+      <c r="D49" s="4">
+        <v>46103</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="F49" s="2">
         <f>2.0024-0.0027</f>
         <v>1.9997000000000003</v>
       </c>
-      <c r="M49" s="9"/>
-      <c r="N49" s="8"/>
+      <c r="G49" s="2">
+        <v>0.50600000000000001</v>
+      </c>
+      <c r="H49" s="3">
+        <v>-6.62</v>
+      </c>
+      <c r="I49" s="2">
+        <v>10.2639</v>
+      </c>
+      <c r="J49" s="2">
+        <v>10.7363</v>
+      </c>
+      <c r="K49" s="2">
+        <v>10.712300000000001</v>
+      </c>
+      <c r="L49" s="2">
+        <f t="shared" si="3"/>
+        <v>5.3523639607491229E-2</v>
+      </c>
+      <c r="M49" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B49, Characterization!A:A, 0))*L49/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B49, Characterization!A:A, 0))*0.01)</f>
+        <v>0.15276133322519878</v>
+      </c>
+      <c r="N49" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B49, Characterization!A:A, 0))*F49</f>
+        <v>7.9805416850377481E-2</v>
+      </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B50" t="s">
         <v>164</v>
@@ -6554,17 +6927,48 @@
       <c r="C50" s="4">
         <v>46100</v>
       </c>
-      <c r="D50" s="4"/>
+      <c r="D50" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F50" s="2">
         <f>2.002-0.0013</f>
         <v>2.0006999999999997</v>
       </c>
-      <c r="M50" s="9"/>
-      <c r="N50" s="8"/>
+      <c r="G50" s="2">
+        <v>0.50039999999999996</v>
+      </c>
+      <c r="H50" s="3">
+        <v>-10.15</v>
+      </c>
+      <c r="I50" s="2">
+        <v>10.7189</v>
+      </c>
+      <c r="J50" s="2">
+        <v>11.2569</v>
+      </c>
+      <c r="K50" s="2">
+        <v>11.2318</v>
+      </c>
+      <c r="L50" s="2">
+        <f t="shared" si="3"/>
+        <v>4.8937414700721611E-2</v>
+      </c>
+      <c r="M50" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B50, Characterization!A:A, 0))*L50/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B50, Characterization!A:A, 0))*0.01)</f>
+        <v>0.11243371027490792</v>
+      </c>
+      <c r="N50" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B50, Characterization!A:A, 0))*F50</f>
+        <v>7.8653977889724017E-2</v>
+      </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B51" t="s">
         <v>164</v>
@@ -6572,17 +6976,48 @@
       <c r="C51" s="4">
         <v>46100</v>
       </c>
-      <c r="D51" s="4"/>
+      <c r="D51" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F51" s="2">
         <f>2.0021-0.0009</f>
         <v>2.0011999999999999</v>
       </c>
-      <c r="M51" s="9"/>
-      <c r="N51" s="8"/>
+      <c r="G51" s="2">
+        <v>0.49659999999999999</v>
+      </c>
+      <c r="H51" s="3">
+        <v>-8.5500000000000007</v>
+      </c>
+      <c r="I51" s="2">
+        <v>10.160600000000001</v>
+      </c>
+      <c r="J51" s="2">
+        <v>10.7181</v>
+      </c>
+      <c r="K51" s="2">
+        <v>10.695499999999999</v>
+      </c>
+      <c r="L51" s="2">
+        <f t="shared" si="3"/>
+        <v>4.2250888016452944E-2</v>
+      </c>
+      <c r="M51" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B51, Characterization!A:A, 0))*L51/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B51, Characterization!A:A, 0))*0.01)</f>
+        <v>9.7071415217800661E-2</v>
+      </c>
+      <c r="N51" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B51, Characterization!A:A, 0))*F51</f>
+        <v>7.8673634504381321E-2</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B52" t="s">
         <v>164</v>
@@ -6590,17 +7025,48 @@
       <c r="C52" s="4">
         <v>46100</v>
       </c>
-      <c r="D52" s="4"/>
+      <c r="D52" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F52" s="2">
         <f>2.0036-0.0017</f>
         <v>2.0019</v>
       </c>
-      <c r="M52" s="9"/>
-      <c r="N52" s="8"/>
+      <c r="G52" s="2">
+        <v>0.505</v>
+      </c>
+      <c r="H52" s="3">
+        <v>-13.67</v>
+      </c>
+      <c r="I52" s="2">
+        <v>9.7448999999999995</v>
+      </c>
+      <c r="J52" s="2">
+        <v>10.3002</v>
+      </c>
+      <c r="K52" s="2">
+        <v>10.2784</v>
+      </c>
+      <c r="L52" s="2">
+        <f t="shared" si="3"/>
+        <v>4.0862230552953523E-2</v>
+      </c>
+      <c r="M52" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B52, Characterization!A:A, 0))*L52/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B52, Characterization!A:A, 0))*0.01)</f>
+        <v>9.3880974695410735E-2</v>
+      </c>
+      <c r="N52" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B52, Characterization!A:A, 0))*F52</f>
+        <v>7.8701153764901555E-2</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B53" t="s">
         <v>164</v>
@@ -6608,17 +7074,48 @@
       <c r="C53" s="4">
         <v>46100</v>
       </c>
-      <c r="D53" s="4"/>
+      <c r="D53" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F53" s="2">
         <f>2.0085-0.0019</f>
         <v>2.0066000000000002</v>
       </c>
-      <c r="M53" s="9"/>
-      <c r="N53" s="8"/>
+      <c r="G53" s="2">
+        <v>0.50249999999999995</v>
+      </c>
+      <c r="H53" s="3">
+        <v>-1.51</v>
+      </c>
+      <c r="I53" s="2">
+        <v>10.650399999999999</v>
+      </c>
+      <c r="J53" s="2">
+        <v>11.274800000000001</v>
+      </c>
+      <c r="K53" s="2">
+        <v>11.228199999999999</v>
+      </c>
+      <c r="L53" s="2">
+        <f t="shared" si="3"/>
+        <v>8.0650744202148739E-2</v>
+      </c>
+      <c r="M53" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B53, Characterization!A:A, 0))*L53/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B53, Characterization!A:A, 0))*0.01)</f>
+        <v>0.18529508480443677</v>
+      </c>
+      <c r="N53" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B53, Characterization!A:A, 0))*F53</f>
+        <v>7.8885925942680193E-2</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B54" t="s">
         <v>164</v>
@@ -6626,17 +7123,48 @@
       <c r="C54" s="4">
         <v>46100</v>
       </c>
-      <c r="D54" s="4"/>
+      <c r="D54" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F54" s="2">
         <f>2.0032-0.0025</f>
         <v>2.0007000000000001</v>
       </c>
-      <c r="M54" s="9"/>
-      <c r="N54" s="8"/>
+      <c r="G54" s="2">
+        <v>0.51490000000000002</v>
+      </c>
+      <c r="H54" s="3">
+        <v>-1.62</v>
+      </c>
+      <c r="I54" s="2">
+        <v>10.289199999999999</v>
+      </c>
+      <c r="J54" s="2">
+        <v>10.752800000000001</v>
+      </c>
+      <c r="K54" s="2">
+        <v>10.7179</v>
+      </c>
+      <c r="L54" s="2">
+        <f t="shared" si="3"/>
+        <v>8.1408910660135989E-2</v>
+      </c>
+      <c r="M54" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B54, Characterization!A:A, 0))*L54/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B54, Characterization!A:A, 0))*0.01)</f>
+        <v>0.18703697224166249</v>
+      </c>
+      <c r="N54" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B54, Characterization!A:A, 0))*F54</f>
+        <v>7.865397788972403E-2</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B55" t="s">
         <v>164</v>
@@ -6644,85 +7172,335 @@
       <c r="C55" s="4">
         <v>46100</v>
       </c>
-      <c r="D55" s="4"/>
+      <c r="D55" s="4">
+        <v>46106</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="F55" s="2">
         <f>2.0021-0.0037</f>
         <v>1.9984</v>
       </c>
-      <c r="M55" s="9"/>
-      <c r="N55" s="8"/>
+      <c r="G55" s="2">
+        <v>0.503</v>
+      </c>
+      <c r="H55" s="3">
+        <v>-2.11</v>
+      </c>
+      <c r="I55" s="2">
+        <v>10.1212</v>
+      </c>
+      <c r="J55" s="2">
+        <v>10.7133</v>
+      </c>
+      <c r="K55" s="2">
+        <v>10.6708</v>
+      </c>
+      <c r="L55" s="2">
+        <f t="shared" si="3"/>
+        <v>7.7328966521107059E-2</v>
+      </c>
+      <c r="M55" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B55, Characterization!A:A, 0))*L55/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B55, Characterization!A:A, 0))*0.01)</f>
+        <v>0.17766330058224353</v>
+      </c>
+      <c r="N55" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B55, Characterization!A:A, 0))*F55</f>
+        <v>7.856355746230044E-2</v>
+      </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B56" t="s">
         <v>162</v>
       </c>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="M56" s="9"/>
-      <c r="N56" s="8"/>
+      <c r="C56" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D56" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F56" s="2">
+        <f>2.0024-0.0023</f>
+        <v>2.0001000000000002</v>
+      </c>
+      <c r="G56" s="2">
+        <v>0.49709999999999999</v>
+      </c>
+      <c r="H56" s="3">
+        <v>-28.37</v>
+      </c>
+      <c r="I56" s="2">
+        <v>10.866300000000001</v>
+      </c>
+      <c r="J56" s="2">
+        <v>11.392099999999999</v>
+      </c>
+      <c r="K56" s="2">
+        <v>11.373100000000001</v>
+      </c>
+      <c r="L56" s="2">
+        <f t="shared" si="3"/>
+        <v>3.7490134175213782E-2</v>
+      </c>
+      <c r="M56" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B56, Characterization!A:A, 0))*L56/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B56, Characterization!A:A, 0))*0.01)</f>
+        <v>0.10795454545453606</v>
+      </c>
+      <c r="N56" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B56, Characterization!A:A, 0))*F56</f>
+        <v>8.1511950488862395E-2</v>
+      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B57" t="s">
         <v>162</v>
       </c>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="M57" s="9"/>
-      <c r="N57" s="8"/>
+      <c r="C57" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D57" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F57" s="2">
+        <f>2.0038-0.0042</f>
+        <v>1.9996</v>
+      </c>
+      <c r="G57" s="2">
+        <v>0.49809999999999999</v>
+      </c>
+      <c r="H57" s="3">
+        <v>-40.17</v>
+      </c>
+      <c r="I57" s="2">
+        <v>10.8736</v>
+      </c>
+      <c r="J57" s="2">
+        <v>11.370699999999999</v>
+      </c>
+      <c r="K57" s="2">
+        <v>11.3551</v>
+      </c>
+      <c r="L57" s="2">
+        <f t="shared" si="3"/>
+        <v>3.2398753894079244E-2</v>
+      </c>
+      <c r="M57" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B57, Characterization!A:A, 0))*L57/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B57, Characterization!A:A, 0))*0.01)</f>
+        <v>9.3293684508632735E-2</v>
+      </c>
+      <c r="N57" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B57, Characterization!A:A, 0))*F57</f>
+        <v>8.1491573520088623E-2</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B58" t="s">
         <v>162</v>
       </c>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="M58" s="9"/>
-      <c r="N58" s="8"/>
+      <c r="C58" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D58" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F58" s="2">
+        <f>2.0081-0.0025</f>
+        <v>2.0056000000000003</v>
+      </c>
+      <c r="H58" s="3">
+        <v>-43.07</v>
+      </c>
+      <c r="I58" s="2">
+        <v>10.099600000000001</v>
+      </c>
+      <c r="J58" s="2">
+        <v>10.6029</v>
+      </c>
+      <c r="K58" s="2">
+        <v>10.5863</v>
+      </c>
+      <c r="L58" s="2">
+        <f t="shared" si="3"/>
+        <v>3.4107252927882525E-2</v>
+      </c>
+      <c r="M58" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B58, Characterization!A:A, 0))*L58/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B58, Characterization!A:A, 0))*0.01)</f>
+        <v>9.8213385135516279E-2</v>
+      </c>
+      <c r="N58" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B58, Characterization!A:A, 0))*F58</f>
+        <v>8.1736097145373957E-2</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B59" t="s">
         <v>162</v>
       </c>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="M59" s="9"/>
-      <c r="N59" s="8"/>
+      <c r="C59" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D59" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F59" s="2">
+        <f>2.0044-0.0019</f>
+        <v>2.0024999999999999</v>
+      </c>
+      <c r="G59" s="2">
+        <v>0.51390000000000002</v>
+      </c>
+      <c r="H59" s="3">
+        <v>-5.77</v>
+      </c>
+      <c r="I59" s="2">
+        <v>10.0169</v>
+      </c>
+      <c r="J59" s="2">
+        <v>10.569599999999999</v>
+      </c>
+      <c r="K59" s="2">
+        <v>10.5375</v>
+      </c>
+      <c r="L59" s="2">
+        <f t="shared" si="3"/>
+        <v>6.1659623511332688E-2</v>
+      </c>
+      <c r="M59" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B59, Characterization!A:A, 0))*L59/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B59, Characterization!A:A, 0))*0.01)</f>
+        <v>0.17755168861104209</v>
+      </c>
+      <c r="N59" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B59, Characterization!A:A, 0))*F59</f>
+        <v>8.1609759938976525E-2</v>
+      </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B60" t="s">
         <v>162</v>
       </c>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="M60" s="9"/>
-      <c r="N60" s="8"/>
+      <c r="C60" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D60" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F60" s="2">
+        <f>2.0056-0.003</f>
+        <v>2.0025999999999997</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="H60" s="3">
+        <v>-5.12</v>
+      </c>
+      <c r="I60" s="2">
+        <v>10.1943</v>
+      </c>
+      <c r="J60" s="2">
+        <v>10.7667</v>
+      </c>
+      <c r="K60" s="2">
+        <v>10.734999999999999</v>
+      </c>
+      <c r="L60" s="2">
+        <f t="shared" si="3"/>
+        <v>5.8627704827077437E-2</v>
+      </c>
+      <c r="M60" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B60, Characterization!A:A, 0))*L60/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B60, Characterization!A:A, 0))*0.01)</f>
+        <v>0.16882114094524348</v>
+      </c>
+      <c r="N60" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B60, Characterization!A:A, 0))*F60</f>
+        <v>8.1613835332731269E-2</v>
+      </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B61" t="s">
         <v>162</v>
       </c>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="M61" s="9"/>
-      <c r="N61" s="8"/>
+      <c r="C61" s="4">
+        <v>46101</v>
+      </c>
+      <c r="D61" s="4">
+        <v>46107</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F61" s="2">
+        <f>2.0033-0.0025</f>
+        <v>2.0007999999999999</v>
+      </c>
+      <c r="G61" s="2">
+        <v>0.50649999999999995</v>
+      </c>
+      <c r="H61" s="3">
+        <v>-6.76</v>
+      </c>
+      <c r="I61" s="2">
+        <v>10.203900000000001</v>
+      </c>
+      <c r="J61" s="2">
+        <v>10.795500000000001</v>
+      </c>
+      <c r="K61" s="2">
+        <v>10.7651</v>
+      </c>
+      <c r="L61" s="2">
+        <f t="shared" si="3"/>
+        <v>5.4169636493229208E-2</v>
+      </c>
+      <c r="M61" s="9">
+        <f>INDEX(Characterization!M:M, MATCH('Trial Metadata'!B61, Characterization!A:A, 0))*L61/(INDEX(Characterization!O:O, MATCH('Trial Metadata'!B61, Characterization!A:A, 0))*0.01)</f>
+        <v>0.15598393053845774</v>
+      </c>
+      <c r="N61" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B61, Characterization!A:A, 0))*F61</f>
+        <v>8.1540478245145681E-2</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
@@ -6735,10 +7513,15 @@
       <c r="C62" s="4">
         <v>46031</v>
       </c>
+      <c r="D62" s="4"/>
       <c r="F62" s="2">
         <f>2.0038-0.0083</f>
         <v>1.9955000000000001</v>
       </c>
+      <c r="N62" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B62, Characterization!A:A, 0))*F62</f>
+        <v>9.5923997443002049E-2</v>
+      </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
@@ -6751,10 +7534,15 @@
       <c r="C63" s="4">
         <v>46031</v>
       </c>
+      <c r="D63" s="4"/>
       <c r="F63" s="2">
         <f>2.0063-0.0145</f>
         <v>1.9918</v>
       </c>
+      <c r="N63" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B63, Characterization!A:A, 0))*F63</f>
+        <v>9.5746137863679026E-2</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
@@ -6767,12 +7555,17 @@
       <c r="C64" s="4">
         <v>46031</v>
       </c>
+      <c r="D64" s="4"/>
       <c r="F64" s="2">
         <f>2.0138-0.0145</f>
         <v>1.9992999999999999</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="N64" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B64, Characterization!A:A, 0))*F64</f>
+        <v>9.6106664037982459E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>57</v>
       </c>
@@ -6783,12 +7576,17 @@
       <c r="C65" s="4">
         <v>46031</v>
       </c>
+      <c r="D65" s="4"/>
       <c r="F65" s="2">
         <f>2.0277-0.0147</f>
         <v>2.0129999999999999</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="N65" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B65, Characterization!A:A, 0))*F65</f>
+        <v>9.676522518304341E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>58</v>
       </c>
@@ -6799,12 +7597,17 @@
       <c r="C66" s="4">
         <v>46031</v>
       </c>
+      <c r="D66" s="4"/>
       <c r="F66" s="2">
         <f>2.0169-0.0108</f>
         <v>2.0061</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="N66" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B66, Characterization!A:A, 0))*F66</f>
+        <v>9.6433541102684248E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>59</v>
       </c>
@@ -6815,9 +7618,14 @@
       <c r="C67" s="4">
         <v>46031</v>
       </c>
+      <c r="D67" s="4"/>
       <c r="F67" s="2">
         <f>2.0203-0.0114</f>
         <v>2.0089000000000001</v>
+      </c>
+      <c r="N67" s="8">
+        <f>INDEX(Characterization!S:S, MATCH('Trial Metadata'!B67, Characterization!A:A, 0))*F67</f>
+        <v>9.6568137541090879E-2</v>
       </c>
     </row>
   </sheetData>
@@ -6828,6 +7636,1940 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FB2F3F8-58E1-498C-8CE8-5AC6F1098C32}">
+  <dimension ref="A1:J73"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.453125" style="13" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" customWidth="1"/>
+    <col min="8" max="8" width="23.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" t="s">
+        <v>243</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="H1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D2" t="str">
+        <f>CONCATENATE(ROW(B2)-1,"-",TEXT(B2, "mm-dd-yyyy"),"-",C2)</f>
+        <v>1-07-18-2025-FGF-SF-20-1</v>
+      </c>
+      <c r="E2" t="str">
+        <f>SUBSTITUTE(D2,"-","_")</f>
+        <v>1_07_18_2025_FGF_SF_20_1</v>
+      </c>
+      <c r="F2" s="13">
+        <v>148.1</v>
+      </c>
+      <c r="G2" s="13">
+        <v>149</v>
+      </c>
+      <c r="H2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" t="str">
+        <f t="shared" ref="D3:D66" si="0">CONCATENATE(ROW(B3)-1,"-",TEXT(B3, "mm-dd-yyyy"),"-",C3)</f>
+        <v>2-07-18-2025-FGF-SF-20-2</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E4" si="1">SUBSTITUTE(D3,"-","_")</f>
+        <v>2_07_18_2025_FGF_SF_20_2</v>
+      </c>
+      <c r="F3" s="13">
+        <v>132.69999999999999</v>
+      </c>
+      <c r="G3" s="13">
+        <v>134.30000000000001</v>
+      </c>
+      <c r="I3" t="s">
+        <v>244</v>
+      </c>
+      <c r="J3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" t="str">
+        <f t="shared" si="0"/>
+        <v>3-07-18-2025-FGF-SF-20-3</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="1"/>
+        <v>3_07_18_2025_FGF_SF_20_3</v>
+      </c>
+      <c r="F4" s="13">
+        <v>171.9</v>
+      </c>
+      <c r="G4" s="13">
+        <v>171.6</v>
+      </c>
+      <c r="I4" t="s">
+        <v>244</v>
+      </c>
+      <c r="J4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" t="str">
+        <f t="shared" si="0"/>
+        <v>4-07-22-2025-FGF-RM-20-1</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" ref="E3:E66" si="2">SUBSTITUTE(D5,"-","_")</f>
+        <v>4_07_22_2025_FGF_RM_20_1</v>
+      </c>
+      <c r="F5" s="13">
+        <v>287.7</v>
+      </c>
+      <c r="G5" s="13">
+        <v>276</v>
+      </c>
+      <c r="I5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" t="str">
+        <f t="shared" si="0"/>
+        <v>5-07-22-2025-FGF-RM-20-2</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="2"/>
+        <v>5_07_22_2025_FGF_RM_20_2</v>
+      </c>
+      <c r="F6" s="13">
+        <v>280.7</v>
+      </c>
+      <c r="G6" s="13">
+        <v>458.2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I6" t="s">
+        <v>244</v>
+      </c>
+      <c r="J6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" t="str">
+        <f t="shared" si="0"/>
+        <v>6-07-22-2025-FGF-RM-20-3</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="2"/>
+        <v>6_07_22_2025_FGF_RM_20_3</v>
+      </c>
+      <c r="F7" s="13">
+        <v>271.10000000000002</v>
+      </c>
+      <c r="G7" s="13">
+        <v>323.7</v>
+      </c>
+      <c r="H7" t="s">
+        <v>258</v>
+      </c>
+      <c r="I7" t="s">
+        <v>244</v>
+      </c>
+      <c r="J7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" si="0"/>
+        <v>7-07-18-2025-FGF-CO-20-1</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="2"/>
+        <v>7_07_18_2025_FGF_CO_20_1</v>
+      </c>
+      <c r="F8" s="13">
+        <v>245.2</v>
+      </c>
+      <c r="G8" s="13">
+        <v>540.9</v>
+      </c>
+      <c r="H8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C9" t="s">
+        <v>235</v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="0"/>
+        <v>8-07-18-2025-FGF-CO-20-2</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="2"/>
+        <v>8_07_18_2025_FGF_CO_20_2</v>
+      </c>
+      <c r="F9" s="13">
+        <v>201.9</v>
+      </c>
+      <c r="G9" s="13">
+        <v>180.2</v>
+      </c>
+      <c r="H9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12">
+        <v>45856</v>
+      </c>
+      <c r="C10" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10" t="str">
+        <f t="shared" si="0"/>
+        <v>9-07-18-2025-FGF-CO-20-3</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="2"/>
+        <v>9_07_18_2025_FGF_CO_20_3</v>
+      </c>
+      <c r="F10" s="13">
+        <v>182.4</v>
+      </c>
+      <c r="G10" s="13">
+        <v>198.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C11" t="s">
+        <v>209</v>
+      </c>
+      <c r="D11" t="str">
+        <f t="shared" si="0"/>
+        <v>10-07-22-2025-FGF-OR-20-1</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="2"/>
+        <v>10_07_22_2025_FGF_OR_20_1</v>
+      </c>
+      <c r="F11" s="13">
+        <v>197</v>
+      </c>
+      <c r="G11" s="13">
+        <v>186.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C12" t="s">
+        <v>210</v>
+      </c>
+      <c r="D12" t="str">
+        <f t="shared" si="0"/>
+        <v>11-07-22-2025-FGF-OR-20-2</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="2"/>
+        <v>11_07_22_2025_FGF_OR_20_2</v>
+      </c>
+      <c r="F12" s="13">
+        <v>172.2</v>
+      </c>
+      <c r="G12" s="13">
+        <v>212.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="12">
+        <v>45860</v>
+      </c>
+      <c r="C13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" t="str">
+        <f t="shared" si="0"/>
+        <v>12-07-22-2025-FGF-OR-20-3</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="2"/>
+        <v>12_07_22_2025_FGF_OR_20_3</v>
+      </c>
+      <c r="F13" s="13">
+        <v>246.1</v>
+      </c>
+      <c r="G13" s="13">
+        <v>230.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C14" t="s">
+        <v>212</v>
+      </c>
+      <c r="D14" t="str">
+        <f t="shared" si="0"/>
+        <v>13-07-24-2025-FGF-SOD-20-1</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="2"/>
+        <v>13_07_24_2025_FGF_SOD_20_1</v>
+      </c>
+      <c r="F14" s="13">
+        <v>619.79999999999995</v>
+      </c>
+      <c r="G14" s="13">
+        <v>1009.2</v>
+      </c>
+      <c r="H14" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C15" t="s">
+        <v>213</v>
+      </c>
+      <c r="D15" t="str">
+        <f t="shared" si="0"/>
+        <v>14-07-24-2025-FGF-SOD-20-2</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="2"/>
+        <v>14_07_24_2025_FGF_SOD_20_2</v>
+      </c>
+      <c r="F15" s="13">
+        <v>671.8</v>
+      </c>
+      <c r="G15" s="13">
+        <v>1344.7</v>
+      </c>
+      <c r="H15" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C16" t="s">
+        <v>214</v>
+      </c>
+      <c r="D16" t="str">
+        <f t="shared" si="0"/>
+        <v>15-07-24-2025-FGF-SOD-20-3</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="2"/>
+        <v>15_07_24_2025_FGF_SOD_20_3</v>
+      </c>
+      <c r="F16" s="13">
+        <v>580.20000000000005</v>
+      </c>
+      <c r="G16" s="13">
+        <v>1153.9000000000001</v>
+      </c>
+      <c r="H16" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C17" t="s">
+        <v>215</v>
+      </c>
+      <c r="D17" t="str">
+        <f t="shared" si="0"/>
+        <v>16-07-30-2026-MF-AS-20-1</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="2"/>
+        <v>16_07_30_2026_MF_AS_20_1</v>
+      </c>
+      <c r="F17" s="13">
+        <v>97.8</v>
+      </c>
+      <c r="G17" s="13">
+        <v>96.6</v>
+      </c>
+      <c r="H17" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D18" t="str">
+        <f t="shared" si="0"/>
+        <v>17-07-30-2026-MF-AS-20-2</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="2"/>
+        <v>17_07_30_2026_MF_AS_20_2</v>
+      </c>
+      <c r="F18" s="13">
+        <v>143</v>
+      </c>
+      <c r="G18" s="13">
+        <v>275.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D19" t="str">
+        <f t="shared" si="0"/>
+        <v>18-07-30-2026-MF-AS-20-3</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="2"/>
+        <v>18_07_30_2026_MF_AS_20_3</v>
+      </c>
+      <c r="F19" s="13">
+        <v>149.80000000000001</v>
+      </c>
+      <c r="G19" s="13">
+        <v>149.30000000000001</v>
+      </c>
+      <c r="H19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C20" t="s">
+        <v>218</v>
+      </c>
+      <c r="D20" t="str">
+        <f t="shared" si="0"/>
+        <v>19-07-24-2025-FGF-BW-20-1</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="2"/>
+        <v>19_07_24_2025_FGF_BW_20_1</v>
+      </c>
+      <c r="F20" s="13">
+        <v>207.9</v>
+      </c>
+      <c r="G20" s="13">
+        <v>284.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C21" t="s">
+        <v>219</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" si="0"/>
+        <v>20-07-24-2025-FGF-BW-20-2</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="2"/>
+        <v>20_07_24_2025_FGF_BW_20_2</v>
+      </c>
+      <c r="F21" s="13">
+        <v>263.60000000000002</v>
+      </c>
+      <c r="G21" s="13">
+        <v>561.20000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12">
+        <v>45862</v>
+      </c>
+      <c r="C22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D22" t="str">
+        <f t="shared" si="0"/>
+        <v>21-07-24-2025-FGF-BW-20-3</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="2"/>
+        <v>21_07_24_2025_FGF_BW_20_3</v>
+      </c>
+      <c r="F22" s="13">
+        <v>226.5</v>
+      </c>
+      <c r="G22" s="13">
+        <v>239.7</v>
+      </c>
+      <c r="H22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C23" t="s">
+        <v>221</v>
+      </c>
+      <c r="D23" t="str">
+        <f t="shared" si="0"/>
+        <v>22-07-30-2026-MF-CH-20-1</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="2"/>
+        <v>22_07_30_2026_MF_CH_20_1</v>
+      </c>
+      <c r="F23" s="13">
+        <v>62.1</v>
+      </c>
+      <c r="G23" s="13">
+        <v>59.7</v>
+      </c>
+      <c r="H23" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C24" t="s">
+        <v>222</v>
+      </c>
+      <c r="D24" t="str">
+        <f t="shared" si="0"/>
+        <v>23-07-30-2026-MF-CH-20-2</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="2"/>
+        <v>23_07_30_2026_MF_CH_20_2</v>
+      </c>
+      <c r="F24" s="13">
+        <v>101.7</v>
+      </c>
+      <c r="G24" s="13">
+        <v>140.19999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="12">
+        <v>46233</v>
+      </c>
+      <c r="C25" t="s">
+        <v>223</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="0"/>
+        <v>24-07-30-2026-MF-CH-20-3</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="2"/>
+        <v>24_07_30_2026_MF_CH_20_3</v>
+      </c>
+      <c r="F25" s="13">
+        <v>91.2</v>
+      </c>
+      <c r="G25" s="13">
+        <v>94.2</v>
+      </c>
+      <c r="H25" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" t="str">
+        <f t="shared" si="0"/>
+        <v>25-03-09-2026-Soy-UD-15-1</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="2"/>
+        <v>25_03_09_2026_Soy_UD_15_1</v>
+      </c>
+      <c r="F26" s="13">
+        <v>447.4</v>
+      </c>
+      <c r="G26" s="13">
+        <v>637.29999999999995</v>
+      </c>
+      <c r="H26" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" t="str">
+        <f t="shared" si="0"/>
+        <v>26-03-09-2026-Soy-UD-15-2</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="2"/>
+        <v>26_03_09_2026_Soy_UD_15_2</v>
+      </c>
+      <c r="F27" s="13">
+        <v>574.70000000000005</v>
+      </c>
+      <c r="G27" s="13">
+        <v>564.20000000000005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C28" t="s">
+        <v>224</v>
+      </c>
+      <c r="D28" t="str">
+        <f t="shared" si="0"/>
+        <v>27-03-09-2026-Soy-UD-15-3</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="2"/>
+        <v>27_03_09_2026_Soy_UD_15_3</v>
+      </c>
+      <c r="F28" s="13">
+        <v>453.1</v>
+      </c>
+      <c r="G28" s="13">
+        <v>967.6</v>
+      </c>
+      <c r="H28" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C29" t="s">
+        <v>225</v>
+      </c>
+      <c r="D29" t="str">
+        <f t="shared" si="0"/>
+        <v>28-03-09-2026-Soy-UD-25-1</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="2"/>
+        <v>28_03_09_2026_Soy_UD_25_1</v>
+      </c>
+      <c r="F29" s="13">
+        <v>461.8</v>
+      </c>
+      <c r="G29" s="13">
+        <v>730.2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C30" t="s">
+        <v>226</v>
+      </c>
+      <c r="D30" t="str">
+        <f t="shared" si="0"/>
+        <v>29-03-09-2026-Soy-UD-25-2</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="2"/>
+        <v>29_03_09_2026_Soy_UD_25_2</v>
+      </c>
+      <c r="F30" s="13">
+        <v>348.2</v>
+      </c>
+      <c r="G30" s="13">
+        <v>292</v>
+      </c>
+      <c r="H30" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12">
+        <v>46090</v>
+      </c>
+      <c r="C31" t="s">
+        <v>227</v>
+      </c>
+      <c r="D31" t="str">
+        <f t="shared" si="0"/>
+        <v>30-03-09-2026-Soy-UD-25-3</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="2"/>
+        <v>30_03_09_2026_Soy_UD_25_3</v>
+      </c>
+      <c r="F31" s="13">
+        <v>445.5</v>
+      </c>
+      <c r="G31" s="13">
+        <v>944.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C32" t="s">
+        <v>228</v>
+      </c>
+      <c r="D32" t="str">
+        <f t="shared" si="0"/>
+        <v>31-03-10-2026-Soy-C-15-1</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="2"/>
+        <v>31_03_10_2026_Soy_C_15_1</v>
+      </c>
+      <c r="F32" s="13">
+        <v>133.5</v>
+      </c>
+      <c r="G32" s="13">
+        <v>126.4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C33" t="s">
+        <v>229</v>
+      </c>
+      <c r="D33" t="str">
+        <f t="shared" si="0"/>
+        <v>32-03-10-2026-Soy-C-15-2</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="2"/>
+        <v>32_03_10_2026_Soy_C_15_2</v>
+      </c>
+      <c r="F33" s="13">
+        <v>207.6</v>
+      </c>
+      <c r="G33" s="13">
+        <v>245.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C34" t="s">
+        <v>230</v>
+      </c>
+      <c r="D34" t="str">
+        <f t="shared" si="0"/>
+        <v>33-03-10-2026-Soy-C-15-3</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="2"/>
+        <v>33_03_10_2026_Soy_C_15_3</v>
+      </c>
+      <c r="F34" s="13">
+        <v>169.4</v>
+      </c>
+      <c r="G34" s="13">
+        <v>288.10000000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C35" t="s">
+        <v>231</v>
+      </c>
+      <c r="D35" t="str">
+        <f t="shared" si="0"/>
+        <v>34-03-10-2026-Soy-C-25-1</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="2"/>
+        <v>34_03_10_2026_Soy_C_25_1</v>
+      </c>
+      <c r="F35" s="13">
+        <v>122.5</v>
+      </c>
+      <c r="G35" s="13">
+        <v>108.2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C36" t="s">
+        <v>232</v>
+      </c>
+      <c r="D36" t="str">
+        <f t="shared" si="0"/>
+        <v>35-03-10-2026-Soy-C-25-2</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="2"/>
+        <v>35_03_10_2026_Soy_C_25_2</v>
+      </c>
+      <c r="F36" s="13">
+        <v>173.4</v>
+      </c>
+      <c r="G36" s="13">
+        <v>452.9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" s="12">
+        <v>46091</v>
+      </c>
+      <c r="C37" t="s">
+        <v>233</v>
+      </c>
+      <c r="D37" t="str">
+        <f t="shared" si="0"/>
+        <v>36-03-10-2026-Soy-C-25-3</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" si="2"/>
+        <v>36_03_10_2026_Soy_C_25_3</v>
+      </c>
+      <c r="F37" s="13">
+        <v>163.30000000000001</v>
+      </c>
+      <c r="G37" s="13">
+        <v>150.9</v>
+      </c>
+      <c r="H37" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C38" t="s">
+        <v>153</v>
+      </c>
+      <c r="D38" t="str">
+        <f t="shared" si="0"/>
+        <v>37-03-14-2026-FGF-OR-15-1</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="2"/>
+        <v>37_03_14_2026_FGF_OR_15_1</v>
+      </c>
+      <c r="F38" s="13">
+        <v>274.89999999999998</v>
+      </c>
+      <c r="G38" s="13">
+        <v>337.7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C39" t="s">
+        <v>154</v>
+      </c>
+      <c r="D39" t="str">
+        <f t="shared" si="0"/>
+        <v>38-03-14-2026-FGF-OR-15-2</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="2"/>
+        <v>38_03_14_2026_FGF_OR_15_2</v>
+      </c>
+      <c r="F39" s="13">
+        <v>245.5</v>
+      </c>
+      <c r="G39" s="13">
+        <v>314.7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C40" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" t="str">
+        <f t="shared" si="0"/>
+        <v>39-03-14-2026-FGF-OR-15-3</v>
+      </c>
+      <c r="E40" t="str">
+        <f t="shared" si="2"/>
+        <v>39_03_14_2026_FGF_OR_15_3</v>
+      </c>
+      <c r="F40" s="13">
+        <v>192.7</v>
+      </c>
+      <c r="G40" s="13">
+        <v>250.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C41" t="s">
+        <v>156</v>
+      </c>
+      <c r="D41" t="str">
+        <f t="shared" si="0"/>
+        <v>40-03-14-2026-FGF-OR-25-1</v>
+      </c>
+      <c r="E41" t="str">
+        <f t="shared" si="2"/>
+        <v>40_03_14_2026_FGF_OR_25_1</v>
+      </c>
+      <c r="F41" s="13">
+        <v>225.5</v>
+      </c>
+      <c r="G41" s="13">
+        <v>729.8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C42" t="s">
+        <v>157</v>
+      </c>
+      <c r="D42" t="str">
+        <f t="shared" si="0"/>
+        <v>41-03-14-2026-FGF-OR-25-2</v>
+      </c>
+      <c r="E42" t="str">
+        <f t="shared" si="2"/>
+        <v>41_03_14_2026_FGF_OR_25_2</v>
+      </c>
+      <c r="F42" s="13">
+        <v>258.60000000000002</v>
+      </c>
+      <c r="G42" s="13">
+        <v>416.3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" s="12">
+        <v>46095</v>
+      </c>
+      <c r="C43" t="s">
+        <v>158</v>
+      </c>
+      <c r="D43" t="str">
+        <f t="shared" si="0"/>
+        <v>42-03-14-2026-FGF-OR-25-3</v>
+      </c>
+      <c r="E43" t="str">
+        <f t="shared" si="2"/>
+        <v>42_03_14_2026_FGF_OR_25_3</v>
+      </c>
+      <c r="F43" s="13">
+        <v>237.4</v>
+      </c>
+      <c r="G43" s="13">
+        <v>171.4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C44" t="s">
+        <v>165</v>
+      </c>
+      <c r="D44" t="str">
+        <f t="shared" si="0"/>
+        <v>43-03-15-2026-FGF-RO-15-1</v>
+      </c>
+      <c r="E44" t="str">
+        <f t="shared" si="2"/>
+        <v>43_03_15_2026_FGF_RO_15_1</v>
+      </c>
+      <c r="F44" s="13">
+        <v>142.69999999999999</v>
+      </c>
+      <c r="G44" s="13">
+        <v>141.19999999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C45" t="s">
+        <v>166</v>
+      </c>
+      <c r="D45" t="str">
+        <f t="shared" si="0"/>
+        <v>44-03-15-2026-FGF-RO-15-2</v>
+      </c>
+      <c r="E45" t="str">
+        <f t="shared" si="2"/>
+        <v>44_03_15_2026_FGF_RO_15_2</v>
+      </c>
+      <c r="F45" s="13">
+        <v>144.19999999999999</v>
+      </c>
+      <c r="G45" s="13">
+        <v>139.30000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C46" t="s">
+        <v>167</v>
+      </c>
+      <c r="D46" t="str">
+        <f t="shared" si="0"/>
+        <v>45-03-15-2026-FGF-RO-15-3</v>
+      </c>
+      <c r="E46" t="str">
+        <f t="shared" si="2"/>
+        <v>45_03_15_2026_FGF_RO_15_3</v>
+      </c>
+      <c r="F46" s="13">
+        <v>146.69999999999999</v>
+      </c>
+      <c r="G46" s="13">
+        <v>176.9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C47" t="s">
+        <v>168</v>
+      </c>
+      <c r="D47" t="str">
+        <f t="shared" si="0"/>
+        <v>46-03-15-2026-FGF-RO-25-1</v>
+      </c>
+      <c r="E47" t="str">
+        <f t="shared" si="2"/>
+        <v>46_03_15_2026_FGF_RO_25_1</v>
+      </c>
+      <c r="F47" s="13">
+        <v>223.8</v>
+      </c>
+      <c r="G47" s="13">
+        <v>293.39999999999998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C48" t="s">
+        <v>169</v>
+      </c>
+      <c r="D48" t="str">
+        <f t="shared" si="0"/>
+        <v>47-03-15-2026-FGF-RO-25-2</v>
+      </c>
+      <c r="E48" t="str">
+        <f t="shared" si="2"/>
+        <v>47_03_15_2026_FGF_RO_25_2</v>
+      </c>
+      <c r="F48" s="13">
+        <v>153.69999999999999</v>
+      </c>
+      <c r="G48" s="13">
+        <v>146.6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" s="12">
+        <v>46096</v>
+      </c>
+      <c r="C49" t="s">
+        <v>170</v>
+      </c>
+      <c r="D49" t="str">
+        <f t="shared" si="0"/>
+        <v>48-03-15-2026-FGF-RO-25-3</v>
+      </c>
+      <c r="E49" t="str">
+        <f t="shared" si="2"/>
+        <v>48_03_15_2026_FGF_RO_25_3</v>
+      </c>
+      <c r="F49" s="13">
+        <v>250.2</v>
+      </c>
+      <c r="G49" s="13">
+        <v>204.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C50" t="s">
+        <v>176</v>
+      </c>
+      <c r="D50" t="str">
+        <f t="shared" si="0"/>
+        <v>49-03-18-2026-FGF-SOD-15-1</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="2"/>
+        <v>49_03_18_2026_FGF_SOD_15_1</v>
+      </c>
+      <c r="F50" s="13">
+        <v>483.1</v>
+      </c>
+      <c r="G50" s="13">
+        <v>412.8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C51" t="s">
+        <v>177</v>
+      </c>
+      <c r="D51" t="str">
+        <f t="shared" si="0"/>
+        <v>50-03-18-2026-FGF-SOD-15-2</v>
+      </c>
+      <c r="E51" t="str">
+        <f t="shared" si="2"/>
+        <v>50_03_18_2026_FGF_SOD_15_2</v>
+      </c>
+      <c r="F51" s="13">
+        <v>496.8</v>
+      </c>
+      <c r="G51" s="13">
+        <v>590.79999999999995</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C52" t="s">
+        <v>178</v>
+      </c>
+      <c r="D52" t="str">
+        <f t="shared" si="0"/>
+        <v>51-03-18-2026-FGF-SOD-15-3</v>
+      </c>
+      <c r="E52" t="str">
+        <f t="shared" si="2"/>
+        <v>51_03_18_2026_FGF_SOD_15_3</v>
+      </c>
+      <c r="F52" s="13">
+        <v>478</v>
+      </c>
+      <c r="G52" s="13">
+        <v>470.9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C53" t="s">
+        <v>179</v>
+      </c>
+      <c r="D53" t="str">
+        <f t="shared" si="0"/>
+        <v>52-03-18-2026-FGF-SOD-25-1</v>
+      </c>
+      <c r="E53" t="str">
+        <f t="shared" si="2"/>
+        <v>52_03_18_2026_FGF_SOD_25_1</v>
+      </c>
+      <c r="F53" s="13">
+        <v>494.6</v>
+      </c>
+      <c r="G53" s="13">
+        <v>563.9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C54" t="s">
+        <v>180</v>
+      </c>
+      <c r="D54" t="str">
+        <f t="shared" si="0"/>
+        <v>53-03-18-2026-FGF-SOD-25-2</v>
+      </c>
+      <c r="E54" t="str">
+        <f t="shared" si="2"/>
+        <v>53_03_18_2026_FGF_SOD_25_2</v>
+      </c>
+      <c r="F54" s="13">
+        <v>506</v>
+      </c>
+      <c r="G54" s="13">
+        <v>517.4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" s="12">
+        <v>46099</v>
+      </c>
+      <c r="C55" t="s">
+        <v>181</v>
+      </c>
+      <c r="D55" t="str">
+        <f t="shared" si="0"/>
+        <v>54-03-18-2026-FGF-SOD-25-3</v>
+      </c>
+      <c r="E55" t="str">
+        <f t="shared" si="2"/>
+        <v>54_03_18_2026_FGF_SOD_25_3</v>
+      </c>
+      <c r="F55" s="13">
+        <v>460.1</v>
+      </c>
+      <c r="G55" s="13">
+        <v>466.4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C56" t="s">
+        <v>237</v>
+      </c>
+      <c r="D56" t="str">
+        <f t="shared" si="0"/>
+        <v>55-03-22-2026-FGF-CO-15-1</v>
+      </c>
+      <c r="E56" t="str">
+        <f t="shared" si="2"/>
+        <v>55_03_22_2026_FGF_CO_15_1</v>
+      </c>
+      <c r="F56" s="13">
+        <v>248.6</v>
+      </c>
+      <c r="G56" s="13">
+        <v>238.5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C57" t="s">
+        <v>238</v>
+      </c>
+      <c r="D57" t="str">
+        <f t="shared" si="0"/>
+        <v>56-03-22-2026-FGF-CO-15-2</v>
+      </c>
+      <c r="E57" t="str">
+        <f t="shared" si="2"/>
+        <v>56_03_22_2026_FGF_CO_15_2</v>
+      </c>
+      <c r="F57" s="13">
+        <v>213.7</v>
+      </c>
+      <c r="G57" s="13">
+        <v>197.8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C58" t="s">
+        <v>239</v>
+      </c>
+      <c r="D58" t="str">
+        <f t="shared" si="0"/>
+        <v>57-03-22-2026-FGF-CO-15-3</v>
+      </c>
+      <c r="E58" t="str">
+        <f t="shared" si="2"/>
+        <v>57_03_22_2026_FGF_CO_15_3</v>
+      </c>
+      <c r="F58" s="13">
+        <v>178.1</v>
+      </c>
+      <c r="G58" s="13">
+        <v>168.8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C59" t="s">
+        <v>240</v>
+      </c>
+      <c r="D59" t="str">
+        <f t="shared" si="0"/>
+        <v>58-03-22-2026-FGF-CO-25-1</v>
+      </c>
+      <c r="E59" t="str">
+        <f t="shared" si="2"/>
+        <v>58_03_22_2026_FGF_CO_25_1</v>
+      </c>
+      <c r="F59" s="13">
+        <v>275.5</v>
+      </c>
+      <c r="G59" s="13">
+        <v>294.7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C60" t="s">
+        <v>241</v>
+      </c>
+      <c r="D60" t="str">
+        <f t="shared" si="0"/>
+        <v>59-03-22-2026-FGF-CO-25-2</v>
+      </c>
+      <c r="E60" t="str">
+        <f t="shared" si="2"/>
+        <v>59_03_22_2026_FGF_CO_25_2</v>
+      </c>
+      <c r="F60" s="13">
+        <v>183.3</v>
+      </c>
+      <c r="G60" s="13">
+        <v>174.8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" s="12">
+        <v>46103</v>
+      </c>
+      <c r="C61" t="s">
+        <v>242</v>
+      </c>
+      <c r="D61" t="str">
+        <f t="shared" si="0"/>
+        <v>60-03-22-2026-FGF-CO-25-3</v>
+      </c>
+      <c r="E61" t="str">
+        <f t="shared" si="2"/>
+        <v>60_03_22_2026_FGF_CO_25_3</v>
+      </c>
+      <c r="F61" s="13">
+        <v>248.5</v>
+      </c>
+      <c r="G61" s="13">
+        <v>263.3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C62" t="s">
+        <v>189</v>
+      </c>
+      <c r="D62" t="str">
+        <f t="shared" si="0"/>
+        <v>61-03-25-2026-FGF-FBW-15-1</v>
+      </c>
+      <c r="E62" t="str">
+        <f t="shared" si="2"/>
+        <v>61_03_25_2026_FGF_FBW_15_1</v>
+      </c>
+      <c r="F62" s="13">
+        <v>284</v>
+      </c>
+      <c r="G62" s="13">
+        <v>277.39999999999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C63" t="s">
+        <v>190</v>
+      </c>
+      <c r="D63" t="str">
+        <f t="shared" si="0"/>
+        <v>62-03-25-2026-FGF-FBW-15-2</v>
+      </c>
+      <c r="E63" t="str">
+        <f t="shared" si="2"/>
+        <v>62_03_25_2026_FGF_FBW_15_2</v>
+      </c>
+      <c r="F63" s="13">
+        <v>286.60000000000002</v>
+      </c>
+      <c r="G63" s="13">
+        <v>238.6</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C64" t="s">
+        <v>191</v>
+      </c>
+      <c r="D64" t="str">
+        <f t="shared" si="0"/>
+        <v>63-03-25-2026-FGF-FBW-15-3</v>
+      </c>
+      <c r="E64" t="str">
+        <f t="shared" si="2"/>
+        <v>63_03_25_2026_FGF_FBW_15_3</v>
+      </c>
+      <c r="F64" s="13">
+        <v>195.9</v>
+      </c>
+      <c r="G64" s="13">
+        <v>184.1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C65" t="s">
+        <v>192</v>
+      </c>
+      <c r="D65" t="str">
+        <f t="shared" si="0"/>
+        <v>64-03-25-2026-FGF-FBW-25-1</v>
+      </c>
+      <c r="E65" t="str">
+        <f t="shared" si="2"/>
+        <v>64_03_25_2026_FGF_FBW_25_1</v>
+      </c>
+      <c r="F65" s="13">
+        <v>175.7</v>
+      </c>
+      <c r="G65" s="13">
+        <v>170.7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C66" t="s">
+        <v>193</v>
+      </c>
+      <c r="D66" t="str">
+        <f t="shared" si="0"/>
+        <v>65-03-25-2026-FGF-FBW-25-2</v>
+      </c>
+      <c r="E66" t="str">
+        <f t="shared" si="2"/>
+        <v>65_03_25_2026_FGF_FBW_25_2</v>
+      </c>
+      <c r="F66" s="13">
+        <v>112.4</v>
+      </c>
+      <c r="G66" s="13">
+        <v>115.6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" s="12">
+        <v>46106</v>
+      </c>
+      <c r="C67" t="s">
+        <v>194</v>
+      </c>
+      <c r="D67" t="str">
+        <f t="shared" ref="D67:D73" si="3">CONCATENATE(ROW(B67)-1,"-",TEXT(B67, "mm-dd-yyyy"),"-",C67)</f>
+        <v>66-03-25-2026-FGF-FBW-25-3</v>
+      </c>
+      <c r="E67" t="str">
+        <f t="shared" ref="E67:E73" si="4">SUBSTITUTE(D67,"-","_")</f>
+        <v>66_03_25_2026_FGF_FBW_25_3</v>
+      </c>
+      <c r="F67" s="13">
+        <v>187</v>
+      </c>
+      <c r="G67" s="13">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C68" t="s">
+        <v>195</v>
+      </c>
+      <c r="D68" t="str">
+        <f t="shared" si="3"/>
+        <v>67-03-26-2026-FGF-SUN-15-1</v>
+      </c>
+      <c r="E68" t="str">
+        <f t="shared" si="4"/>
+        <v>67_03_26_2026_FGF_SUN_15_1</v>
+      </c>
+      <c r="F68" s="13">
+        <v>135.69999999999999</v>
+      </c>
+      <c r="G68" s="13">
+        <v>175.9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C69" t="s">
+        <v>196</v>
+      </c>
+      <c r="D69" t="str">
+        <f t="shared" si="3"/>
+        <v>68-03-26-2026-FGF-SUN-15-2</v>
+      </c>
+      <c r="E69" t="str">
+        <f t="shared" si="4"/>
+        <v>68_03_26_2026_FGF_SUN_15_2</v>
+      </c>
+      <c r="F69" s="13">
+        <v>126.2</v>
+      </c>
+      <c r="G69" s="13">
+        <v>112.8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C70" t="s">
+        <v>197</v>
+      </c>
+      <c r="D70" t="str">
+        <f t="shared" si="3"/>
+        <v>69-03-26-2026-FGF-SUN-15-3</v>
+      </c>
+      <c r="E70" t="str">
+        <f t="shared" si="4"/>
+        <v>69_03_26_2026_FGF_SUN_15_3</v>
+      </c>
+      <c r="F70" s="13">
+        <v>107.4</v>
+      </c>
+      <c r="G70" s="13">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C71" t="s">
+        <v>198</v>
+      </c>
+      <c r="D71" t="str">
+        <f t="shared" si="3"/>
+        <v>70-03-26-2026-FGF-SUN-25-1</v>
+      </c>
+      <c r="E71" t="str">
+        <f t="shared" si="4"/>
+        <v>70_03_26_2026_FGF_SUN_25_1</v>
+      </c>
+      <c r="F71" s="13">
+        <v>159.80000000000001</v>
+      </c>
+      <c r="G71" s="13">
+        <v>149.4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C72" t="s">
+        <v>199</v>
+      </c>
+      <c r="D72" t="str">
+        <f t="shared" si="3"/>
+        <v>71-03-26-2026-FGF-SUN-25-2</v>
+      </c>
+      <c r="E72" t="str">
+        <f t="shared" si="4"/>
+        <v>71_03_26_2026_FGF_SUN_25_2</v>
+      </c>
+      <c r="F72" s="13">
+        <v>140.5</v>
+      </c>
+      <c r="G72" s="13">
+        <v>129.4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" s="12">
+        <v>46107</v>
+      </c>
+      <c r="C73" t="s">
+        <v>200</v>
+      </c>
+      <c r="D73" t="str">
+        <f t="shared" si="3"/>
+        <v>72-03-26-2026-FGF-SUN-25-3</v>
+      </c>
+      <c r="E73" t="str">
+        <f t="shared" si="4"/>
+        <v>72_03_26_2026_FGF_SUN_25_3</v>
+      </c>
+      <c r="F73" s="13">
+        <v>189.8</v>
+      </c>
+      <c r="G73" s="13">
+        <v>176.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DCD1671-150A-431B-9802-17D2A2E7407A}">
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7255,7 +9997,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00F465DB-3416-4852-B573-96C6ABA2B1A8}">
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7591,7 +10333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DF4ED8B-9D6A-4DCD-8C9F-6E04025006A7}">
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7881,7 +10623,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD63824-F95F-4A24-9AAE-5CBB9DC71786}">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>